<commit_message>
feat: add project history outputs and project fields
</commit_message>
<xml_diff>
--- a/templates/项目资料导入模板.xlsx
+++ b/templates/项目资料导入模板.xlsx
@@ -7,7 +7,7 @@
     <sheet name="填写说明" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'导入数据'!A1:AK1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'导入数据'!A1:AP1</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,45 +401,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK1"/>
+  <dimension ref="A1:AP1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="12.83203125" customWidth="1"/>
     <col min="12" max="12" width="12.83203125" customWidth="1"/>
     <col min="13" max="13" width="12.83203125" customWidth="1"/>
     <col min="14" max="14" width="12.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
     <col min="16" max="16" width="12.83203125" customWidth="1"/>
     <col min="17" max="17" width="12.83203125" customWidth="1"/>
     <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="14.83203125" customWidth="1"/>
-    <col min="20" max="20" width="16.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
     <col min="21" max="21" width="12.83203125" customWidth="1"/>
-    <col min="22" max="22" width="20.83203125" customWidth="1"/>
+    <col min="22" max="22" width="12.83203125" customWidth="1"/>
     <col min="23" max="23" width="12.83203125" customWidth="1"/>
-    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1"/>
     <col min="25" max="25" width="16.83203125" customWidth="1"/>
-    <col min="26" max="26" width="16.83203125" customWidth="1"/>
-    <col min="27" max="27" width="16.83203125" customWidth="1"/>
-    <col min="28" max="28" width="16.83203125" customWidth="1"/>
-    <col min="29" max="29" width="16.83203125" customWidth="1"/>
-    <col min="30" max="30" width="20.83203125" customWidth="1"/>
-    <col min="31" max="31" width="12.83203125" customWidth="1"/>
-    <col min="32" max="32" width="12.83203125" customWidth="1"/>
-    <col min="33" max="33" width="12.83203125" customWidth="1"/>
-    <col min="34" max="34" width="12.83203125" customWidth="1"/>
+    <col min="26" max="26" width="12.83203125" customWidth="1"/>
+    <col min="27" max="27" width="20.83203125" customWidth="1"/>
+    <col min="28" max="28" width="12.83203125" customWidth="1"/>
+    <col min="29" max="29" width="12.83203125" customWidth="1"/>
+    <col min="30" max="30" width="12.83203125" customWidth="1"/>
+    <col min="31" max="31" width="16.83203125" customWidth="1"/>
+    <col min="32" max="32" width="16.83203125" customWidth="1"/>
+    <col min="33" max="33" width="16.83203125" customWidth="1"/>
+    <col min="34" max="34" width="16.83203125" customWidth="1"/>
     <col min="35" max="35" width="16.83203125" customWidth="1"/>
-    <col min="36" max="36" width="14.83203125" customWidth="1"/>
+    <col min="36" max="36" width="20.83203125" customWidth="1"/>
     <col min="37" max="37" width="12.83203125" customWidth="1"/>
+    <col min="38" max="38" width="12.83203125" customWidth="1"/>
+    <col min="39" max="39" width="12.83203125" customWidth="1"/>
+    <col min="40" max="40" width="16.83203125" customWidth="1"/>
+    <col min="41" max="41" width="14.83203125" customWidth="1"/>
+    <col min="42" max="42" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,119 +458,134 @@
         <v>优先级</v>
       </c>
       <c r="D1" t="str">
-        <v>集数/场/镜头</v>
+        <v>项目类型</v>
       </c>
       <c r="E1" t="str">
+        <v>制作要求</v>
+      </c>
+      <c r="F1" t="str">
+        <v>场数</v>
+      </c>
+      <c r="G1" t="str">
+        <v>集数</v>
+      </c>
+      <c r="H1" t="str">
         <v>总时长</v>
       </c>
-      <c r="F1" t="str">
+      <c r="I1" t="str">
+        <v>结算情况</v>
+      </c>
+      <c r="J1" t="str">
+        <v>测试结果</v>
+      </c>
+      <c r="K1" t="str">
         <v>项目概述</v>
       </c>
-      <c r="G1" t="str">
+      <c r="L1" t="str">
         <v>引入人员</v>
       </c>
-      <c r="H1" t="str">
+      <c r="M1" t="str">
         <v>接单时间</v>
       </c>
-      <c r="I1" t="str">
+      <c r="N1" t="str">
         <v>客户企业</v>
       </c>
-      <c r="J1" t="str">
+      <c r="O1" t="str">
         <v>客户对接人</v>
       </c>
-      <c r="K1" t="str">
+      <c r="P1" t="str">
         <v>DDL</v>
       </c>
-      <c r="L1" t="str">
+      <c r="Q1" t="str">
         <v>项目状态</v>
       </c>
-      <c r="M1" t="str">
+      <c r="R1" t="str">
         <v>剧本</v>
       </c>
-      <c r="N1" t="str">
+      <c r="S1" t="str">
         <v>故事大纲</v>
       </c>
-      <c r="O1" t="str">
+      <c r="T1" t="str">
         <v>人物小传</v>
       </c>
-      <c r="P1" t="str">
+      <c r="U1" t="str">
         <v>目标参考</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="V1" t="str">
         <v>验收标准</v>
       </c>
-      <c r="R1" t="str">
+      <c r="W1" t="str">
         <v>美术参考</v>
       </c>
-      <c r="S1" t="str">
+      <c r="X1" t="str">
         <v>项目总进度</v>
       </c>
-      <c r="T1" t="str">
+      <c r="Y1" t="str">
         <v>本月完成进度</v>
       </c>
-      <c r="U1" t="str">
+      <c r="Z1" t="str">
         <v>上月进度</v>
       </c>
-      <c r="V1" t="str">
+      <c r="AA1" t="str">
         <v>项目负责人/导演</v>
       </c>
-      <c r="W1" t="str">
+      <c r="AB1" t="str">
+        <v>编导</v>
+      </c>
+      <c r="AC1" t="str">
         <v>PM</v>
       </c>
-      <c r="X1" t="str">
+      <c r="AD1" t="str">
         <v>美术监制</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AE1" t="str">
         <v>视频制作人员</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AF1" t="str">
         <v>资产制作人员</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AG1" t="str">
         <v>资产制作进度</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AH1" t="str">
         <v>资产完成日期</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AI1" t="str">
         <v>视频制作进度</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AJ1" t="str">
         <v>视频制作完成日期</v>
       </c>
-      <c r="AE1" t="str">
+      <c r="AK1" t="str">
         <v>内审情况</v>
       </c>
-      <c r="AF1" t="str">
+      <c r="AL1" t="str">
         <v>其它支持</v>
       </c>
-      <c r="AG1" t="str">
+      <c r="AM1" t="str">
         <v>SVN</v>
       </c>
-      <c r="AH1" t="str">
-        <v>项目地址</v>
-      </c>
-      <c r="AI1" t="str">
+      <c r="AN1" t="str">
         <v>项目表单链接</v>
       </c>
-      <c r="AJ1" t="str">
+      <c r="AO1" t="str">
         <v>风险/阻塞</v>
       </c>
-      <c r="AK1" t="str">
+      <c r="AP1" t="str">
         <v>备注</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK1"/>
+  <autoFilter ref="A1:AP1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AK1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AP1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="95.83203125" customWidth="1"/>
@@ -597,55 +617,87 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>项目状态</v>
+        <v>项目类型</v>
       </c>
       <c r="B4" t="str">
-        <v>可填写：待启动、制作中、资产制作中、资产制作完成、视频制作中、视频制作完成、反馈修改中、待验收、暂停、已完成、已取消。</v>
+        <v>填写：测试项目、正式合作项目。测试项目应同时填写测试结果。</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>人员字段</v>
+        <v>制作要求</v>
       </c>
       <c r="B5" t="str">
-        <v>项目负责人/导演、PM、美术监制、视频制作人员、资产制作人员五个核心岗位均至少填写 1 人，也可填写多人；多人用顿号分隔。</v>
+        <v>填写：片段制作、剧集制作、全片制作。片段/全片填写场数，剧集制作填写集数。</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>产能释放规则</v>
+        <v>结算情况</v>
       </c>
       <c r="B6" t="str">
-        <v>资产制作完成后资产制作人员自动释放；项目负责人/导演和视频制作人员直到项目已完成才释放。</v>
+        <v>填写：损稿、客户撤稿、正常结算、部分结算。</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>剧本等资料</v>
+        <v>测试结果</v>
       </c>
       <c r="B7" t="str">
-        <v>可填写内容摘要，也可填写本地文件或文件夹路径。软件离线运行，不会上传这些内容。</v>
+        <v>仅测试项目填写：测试通过、测试未通过、转正式合作、待定。</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>进度字段</v>
+        <v>项目状态</v>
       </c>
       <c r="B8" t="str">
-        <v>填写 0-100 的数字，不要输入百分号。</v>
+        <v>可填写：待启动、制作中、资产制作中、资产制作完成、视频制作中、视频制作完成、反馈修改中、待验收、暂停、已完成、已取消。</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>人员字段</v>
+      </c>
+      <c r="B9" t="str">
+        <v>项目负责人/导演、编导、PM、美术监制、视频制作人员、资产制作人员均支持多人，多人用顿号分隔；编导可缺省，有导演时美术监制也可缺省。</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>产能释放规则</v>
+      </c>
+      <c r="B10" t="str">
+        <v>资产制作完成后资产制作人员自动释放；项目负责人/导演和视频制作人员直到项目已完成才释放。</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>剧本等资料</v>
+      </c>
+      <c r="B11" t="str">
+        <v>可填写内容摘要，也可填写本地文件或文件夹路径。软件离线运行，不会上传这些内容。</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>进度字段</v>
+      </c>
+      <c r="B12" t="str">
+        <v>填写 0-100 的数字，不要输入百分号。</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>通用规则</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B13" t="str">
         <v>请勿修改第一行表头；一行代表一条记录；人员项目占用百分比允许合计超过 100%，软件会标记为超负荷。</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add project start filters and staffing eligibility
</commit_message>
<xml_diff>
--- a/templates/项目资料导入模板.xlsx
+++ b/templates/项目资料导入模板.xlsx
@@ -7,7 +7,7 @@
     <sheet name="填写说明" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'导入数据'!A1:AP1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'导入数据'!A1:AQ1</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AP1"/>
+  <dimension ref="A1:AQ1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -417,8 +417,8 @@
     <col min="12" max="12" width="12.83203125" customWidth="1"/>
     <col min="13" max="13" width="12.83203125" customWidth="1"/>
     <col min="14" max="14" width="12.83203125" customWidth="1"/>
-    <col min="15" max="15" width="14.83203125" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
     <col min="17" max="17" width="12.83203125" customWidth="1"/>
     <col min="18" max="18" width="12.83203125" customWidth="1"/>
     <col min="19" max="19" width="12.83203125" customWidth="1"/>
@@ -426,25 +426,26 @@
     <col min="21" max="21" width="12.83203125" customWidth="1"/>
     <col min="22" max="22" width="12.83203125" customWidth="1"/>
     <col min="23" max="23" width="12.83203125" customWidth="1"/>
-    <col min="24" max="24" width="14.83203125" customWidth="1"/>
-    <col min="25" max="25" width="16.83203125" customWidth="1"/>
-    <col min="26" max="26" width="12.83203125" customWidth="1"/>
-    <col min="27" max="27" width="20.83203125" customWidth="1"/>
-    <col min="28" max="28" width="12.83203125" customWidth="1"/>
+    <col min="24" max="24" width="12.83203125" customWidth="1"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1"/>
+    <col min="26" max="26" width="16.83203125" customWidth="1"/>
+    <col min="27" max="27" width="12.83203125" customWidth="1"/>
+    <col min="28" max="28" width="20.83203125" customWidth="1"/>
     <col min="29" max="29" width="12.83203125" customWidth="1"/>
     <col min="30" max="30" width="12.83203125" customWidth="1"/>
-    <col min="31" max="31" width="16.83203125" customWidth="1"/>
+    <col min="31" max="31" width="12.83203125" customWidth="1"/>
     <col min="32" max="32" width="16.83203125" customWidth="1"/>
     <col min="33" max="33" width="16.83203125" customWidth="1"/>
     <col min="34" max="34" width="16.83203125" customWidth="1"/>
     <col min="35" max="35" width="16.83203125" customWidth="1"/>
-    <col min="36" max="36" width="20.83203125" customWidth="1"/>
-    <col min="37" max="37" width="12.83203125" customWidth="1"/>
+    <col min="36" max="36" width="16.83203125" customWidth="1"/>
+    <col min="37" max="37" width="20.83203125" customWidth="1"/>
     <col min="38" max="38" width="12.83203125" customWidth="1"/>
     <col min="39" max="39" width="12.83203125" customWidth="1"/>
-    <col min="40" max="40" width="16.83203125" customWidth="1"/>
-    <col min="41" max="41" width="14.83203125" customWidth="1"/>
-    <col min="42" max="42" width="12.83203125" customWidth="1"/>
+    <col min="40" max="40" width="12.83203125" customWidth="1"/>
+    <col min="41" max="41" width="16.83203125" customWidth="1"/>
+    <col min="42" max="42" width="14.83203125" customWidth="1"/>
+    <col min="43" max="43" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,104 +489,107 @@
         <v>接单时间</v>
       </c>
       <c r="N1" t="str">
+        <v>启动时间</v>
+      </c>
+      <c r="O1" t="str">
         <v>客户企业</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>客户对接人</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>DDL</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>项目状态</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>剧本</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>故事大纲</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>人物小传</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>目标参考</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>验收标准</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>美术参考</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>项目总进度</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>本月完成进度</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>上月进度</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>项目负责人/导演</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>编导</v>
       </c>
-      <c r="AC1" t="str">
+      <c r="AD1" t="str">
         <v>PM</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AE1" t="str">
         <v>美术监制</v>
       </c>
-      <c r="AE1" t="str">
+      <c r="AF1" t="str">
         <v>视频制作人员</v>
       </c>
-      <c r="AF1" t="str">
+      <c r="AG1" t="str">
         <v>资产制作人员</v>
       </c>
-      <c r="AG1" t="str">
+      <c r="AH1" t="str">
         <v>资产制作进度</v>
       </c>
-      <c r="AH1" t="str">
+      <c r="AI1" t="str">
         <v>资产完成日期</v>
       </c>
-      <c r="AI1" t="str">
+      <c r="AJ1" t="str">
         <v>视频制作进度</v>
       </c>
-      <c r="AJ1" t="str">
+      <c r="AK1" t="str">
         <v>视频制作完成日期</v>
       </c>
-      <c r="AK1" t="str">
+      <c r="AL1" t="str">
         <v>内审情况</v>
       </c>
-      <c r="AL1" t="str">
+      <c r="AM1" t="str">
         <v>其它支持</v>
       </c>
-      <c r="AM1" t="str">
+      <c r="AN1" t="str">
         <v>SVN</v>
       </c>
-      <c r="AN1" t="str">
+      <c r="AO1" t="str">
         <v>项目表单链接</v>
       </c>
-      <c r="AO1" t="str">
+      <c r="AP1" t="str">
         <v>风险/阻塞</v>
       </c>
-      <c r="AP1" t="str">
+      <c r="AQ1" t="str">
         <v>备注</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP1"/>
+  <autoFilter ref="A1:AQ1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AP1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AQ1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="95.83203125" customWidth="1"/>
@@ -625,79 +629,87 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>制作要求</v>
+        <v>启动时间</v>
       </c>
       <c r="B5" t="str">
-        <v>填写：片段制作、剧集制作、全片制作。片段/全片填写场数，剧集制作填写集数。</v>
+        <v>填写项目正式启动日期，用于项目资料库的启动时间起止筛选。</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>结算情况</v>
+        <v>制作要求</v>
       </c>
       <c r="B6" t="str">
-        <v>填写：损稿、客户撤稿、正常结算、部分结算。</v>
+        <v>填写：片段制作、剧集制作、全片制作。片段/全片填写场数，剧集制作填写集数。</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>测试结果</v>
+        <v>结算情况</v>
       </c>
       <c r="B7" t="str">
-        <v>仅测试项目填写：测试通过、测试未通过、转正式合作、待定。</v>
+        <v>填写：损稿、客户撤稿、正常结算、部分结算、不结算。</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>项目状态</v>
+        <v>测试结果</v>
       </c>
       <c r="B8" t="str">
-        <v>可填写：待启动、制作中、资产制作中、资产制作完成、视频制作中、视频制作完成、反馈修改中、待验收、暂停、已完成、已取消。</v>
+        <v>仅测试项目填写：测试通过、测试未通过、转正式合作、待定。</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>人员字段</v>
+        <v>项目状态</v>
       </c>
       <c r="B9" t="str">
-        <v>项目负责人/导演、编导、PM、美术监制、视频制作人员、资产制作人员均支持多人，多人用顿号分隔；编导可缺省，有导演时美术监制也可缺省。</v>
+        <v>可填写：待启动、制作中、资产制作中、资产制作完成、视频制作中、视频制作完成、反馈修改中、待验收、暂停、已完成、已取消。已完成、已完结、已取消项目不产生用人需求。</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>产能释放规则</v>
+        <v>人员字段</v>
       </c>
       <c r="B10" t="str">
-        <v>资产制作完成后资产制作人员自动释放；项目负责人/导演和视频制作人员直到项目已完成才释放。</v>
+        <v>项目负责人/导演、编导、PM、美术监制、视频制作人员、资产制作人员均支持多人，多人用顿号分隔；编导可缺省，有导演时美术监制也可缺省。</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>剧本等资料</v>
+        <v>产能释放规则</v>
       </c>
       <c r="B11" t="str">
-        <v>可填写内容摘要，也可填写本地文件或文件夹路径。软件离线运行，不会上传这些内容。</v>
+        <v>资产制作完成后资产制作人员自动释放；项目负责人/导演和视频制作人员直到项目已完成才释放。</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>进度字段</v>
+        <v>剧本等资料</v>
       </c>
       <c r="B12" t="str">
-        <v>填写 0-100 的数字，不要输入百分号。</v>
+        <v>可填写内容摘要，也可填写本地文件或文件夹路径。软件离线运行，不会上传这些内容。</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
+        <v>进度字段</v>
+      </c>
+      <c r="B13" t="str">
+        <v>填写 0-100 的数字，不要输入百分号。</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
         <v>通用规则</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B14" t="str">
         <v>请勿修改第一行表头；一行代表一条记录；人员项目占用百分比允许合计超过 100%，软件会标记为超负荷。</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>